<commit_message>
se corrige el excel con los cambios que pidió el profesor
</commit_message>
<xml_diff>
--- a/Casos de prueba calculadora impuestos.xlsx
+++ b/Casos de prueba calculadora impuestos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\b12s308\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1bec37564674e377/Documentos/Trabajos - U/calculadora_impuestos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A29A5082-C147-48D4-8B6A-72FB6FB59279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{50868B31-AD29-465F-8FF4-1FD0CAE8337C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{06946C17-4C28-4ABE-B657-4AEA146628FB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DD02F704-9D04-49AA-A06E-3EE7BF9BBD53}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -32,31 +32,46 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
+      <xlwcv:version setVersion="2"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="68">
   <si>
     <t>CASOS NORMALES</t>
   </si>
   <si>
-    <t>Caso de prueba</t>
-  </si>
-  <si>
-    <t>Nombre</t>
-  </si>
-  <si>
-    <t>Datos de entrada</t>
-  </si>
-  <si>
-    <t>Proceso</t>
-  </si>
-  <si>
-    <t>Resultado esperado</t>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Nombre del caso de prueba</t>
+  </si>
+  <si>
+    <t>Objetivo</t>
+  </si>
+  <si>
+    <t>Precondiciones</t>
+  </si>
+  <si>
+    <t>Precio</t>
+  </si>
+  <si>
+    <t>IVA 19%</t>
+  </si>
+  <si>
+    <t>INC</t>
+  </si>
+  <si>
+    <t>Bolsas</t>
+  </si>
+  <si>
+    <t>Cantidad de bolsas</t>
+  </si>
+  <si>
+    <t>Salida esperada</t>
   </si>
   <si>
     <t>CP-01</t>
@@ -65,139 +80,174 @@
     <t>Cálculo de IVA del 19%</t>
   </si>
   <si>
-    <t>Precio: 100000; IVA: 19%</t>
-  </si>
-  <si>
-    <t>Calcular el 19% sobre el precio</t>
-  </si>
-  <si>
-    <t>IVA: 19000; Total: 119000</t>
+    <t>Verificar que el sistema calcule correctamente el IVA del 19%.</t>
+  </si>
+  <si>
+    <t>El sistema permite ingresar precio y seleccionar impuesto.</t>
+  </si>
+  <si>
+    <t>Sí</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>IVA = 19000; Bolsas = 0; Total = 119000</t>
   </si>
   <si>
     <t>CP-02</t>
   </si>
   <si>
-    <t>Producto con INC</t>
-  </si>
-  <si>
-    <t>Precio: 40000; INC: 8%</t>
-  </si>
-  <si>
-    <t>Calcular el 8% sobre el precio</t>
-  </si>
-  <si>
-    <t>INC: 3200; Total: 43200</t>
+    <t>Producto con Impuesto Nacional al Consumo</t>
+  </si>
+  <si>
+    <t>Verificar que el sistema calcule correctamente el INC del 8%.</t>
+  </si>
+  <si>
+    <t>El sistema tiene configurada la tarifa del INC.</t>
+  </si>
+  <si>
+    <t>INC = 3200; Bolsas = 0; Total = 43200</t>
   </si>
   <si>
     <t>CP-03</t>
   </si>
   <si>
-    <t>IVA 19% + bolsas plásticas</t>
-  </si>
-  <si>
-    <t>Precio: 100000; IVA: 19%; Bolsas: 2</t>
-  </si>
-  <si>
-    <t>Calcular IVA y sumar impuesto de bolsas</t>
-  </si>
-  <si>
-    <t>IVA: 19000; Bolsas: 146; Total: 119146</t>
+    <t>IVA 19% + impuesto a bolsas plásticas</t>
+  </si>
+  <si>
+    <t>Verificar que el sistema permita combinar IVA 19% con el impuesto a bolsas.</t>
+  </si>
+  <si>
+    <t>El producto tiene IVA 19% y se entregan bolsas.</t>
+  </si>
+  <si>
+    <t>IVA = 19000; Bolsas = 146; Total = 119146</t>
   </si>
   <si>
     <t>CASOS EXCEPCIONALES</t>
   </si>
   <si>
+    <t>Excluido</t>
+  </si>
+  <si>
     <t>CP-04</t>
   </si>
   <si>
     <t>Precio muy alto</t>
   </si>
   <si>
-    <t>Precio: 999999999; IVA: 19%</t>
-  </si>
-  <si>
-    <t>Calcular el impuesto dentro del límite máximo</t>
-  </si>
-  <si>
-    <t>El sistema calcula correctamente sin errores de desbordamiento</t>
+    <t>Verificar que el sistema procese correctamente un precio cercano al límite máximo.</t>
+  </si>
+  <si>
+    <t>El precio máximo permitido es 1000000000.</t>
+  </si>
+  <si>
+    <t>IVA = 189999999.81; Bolsas = 0; Total = 1189999998.81</t>
   </si>
   <si>
     <t>CP-05</t>
   </si>
   <si>
-    <t>Ningún impuesto seleccionado</t>
-  </si>
-  <si>
-    <t>Precio: 50000; Impuesto: ninguno</t>
-  </si>
-  <si>
-    <t>Intentar realizar el cálculo sin seleccionar categoría</t>
-  </si>
-  <si>
-    <t>El sistema solicita seleccionar una categoría de impuesto</t>
+    <t>Sin impuesto</t>
+  </si>
+  <si>
+    <t>Verificar que el sistema mantenga el precio de un producto exento de impuesto.</t>
+  </si>
+  <si>
+    <t>El producto está marcado como exento.</t>
+  </si>
+  <si>
+    <t>Impuesto = 0; Bolsas = 0; Total = 50000</t>
   </si>
   <si>
     <t>CP-06</t>
   </si>
   <si>
-    <t>Excluido + bolsas plásticas</t>
-  </si>
-  <si>
-    <t>Precio: 40000; Categoría: Excluido; Bolsas: 1</t>
-  </si>
-  <si>
-    <t>Calcular el impuesto de bolsas independientemente de la categoría</t>
-  </si>
-  <si>
-    <t>IVA: 0; Bolsas: 73; Total: 40073</t>
+    <t>Producto excluido + bolsas plásticas</t>
+  </si>
+  <si>
+    <t>Verificar que el impuesto de bolsas se aplique independientemente del estado excluido del producto.</t>
+  </si>
+  <si>
+    <t>El producto está marcado como excluido.</t>
+  </si>
+  <si>
+    <t>Impuesto = 0; Bolsas = 73; Total = 40073</t>
   </si>
   <si>
     <t>CASOS DE ERROR</t>
   </si>
   <si>
+    <t>IVA 5%</t>
+  </si>
+  <si>
     <t>CP-07</t>
   </si>
   <si>
     <t>Precio negativo</t>
   </si>
   <si>
-    <t>Precio: -50000; IVA: 19%</t>
-  </si>
-  <si>
-    <t>Intentar calcular con precio negativo</t>
-  </si>
-  <si>
-    <t>Error: el precio debe ser mayor que cero</t>
+    <t>Verificar que el sistema rechace un precio negativo.</t>
+  </si>
+  <si>
+    <t>El precio debe ser mayor que cero.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Error: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>PrecioInvalidoError</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; no se calcula el total</t>
+    </r>
   </si>
   <si>
     <t>CP-08</t>
   </si>
   <si>
-    <t>Letras en el precio</t>
-  </si>
-  <si>
-    <t>Precio: abc; IVA: 19%</t>
-  </si>
-  <si>
-    <t>Intentar calcular con un precio no numérico</t>
-  </si>
-  <si>
-    <t>Error: el precio debe ser un valor numérico</t>
+    <t>Letras en el campo de precio</t>
+  </si>
+  <si>
+    <t>Verificar que el sistema rechace valores no numéricos.</t>
+  </si>
+  <si>
+    <t>El precio debe ser numérico.</t>
+  </si>
+  <si>
+    <t>abc</t>
   </si>
   <si>
     <t>CP-09</t>
   </si>
   <si>
-    <t>Precio vacío</t>
-  </si>
-  <si>
-    <t>Precio: vacío; IVA: 19%</t>
-  </si>
-  <si>
-    <t>Intentar calcular sin ingresar precio</t>
-  </si>
-  <si>
-    <t>Error: el precio es obligatorio</t>
+    <t>Campo de precio vacío</t>
+  </si>
+  <si>
+    <t>Verificar que el sistema rechace el campo de precio vacío.</t>
+  </si>
+  <si>
+    <t>El precio es obligatorio.</t>
+  </si>
+  <si>
+    <t>Vacío</t>
   </si>
   <si>
     <t>CP-10</t>
@@ -206,20 +256,40 @@
     <t>IVA 5% e IVA 19% simultáneamente</t>
   </si>
   <si>
-    <t>Precio: 100000; IVA: 5% y 19%</t>
-  </si>
-  <si>
-    <t>Intentar seleccionar las dos tarifas de IVA</t>
-  </si>
-  <si>
-    <t>Error: no se pueden seleccionar IVA 5% e IVA 19% al mismo tiempo</t>
+    <t>Verificar que el sistema no permita seleccionar dos tarifas de IVA.</t>
+  </si>
+  <si>
+    <t>Solo se permite una tarifa de IVA por producto.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Error: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ImpuestoInvalidoError</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; no se calcula el total</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -237,11 +307,16 @@
     </font>
     <font>
       <b/>
-      <sz val="13.5"/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -608,22 +683,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E0CD23D-29A8-4DF3-933E-6D6F995B400E}">
-  <dimension ref="A1:E21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F986A90B-3774-4A82-A914-F988DD67BBC4}">
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="30.85546875" customWidth="1"/>
-    <col min="3" max="3" width="51.85546875" customWidth="1"/>
-    <col min="4" max="4" width="42.28515625" customWidth="1"/>
-    <col min="5" max="5" width="27.42578125" customWidth="1"/>
+    <col min="3" max="3" width="49.44140625" customWidth="1"/>
+    <col min="4" max="4" width="37.88671875" customWidth="1"/>
+    <col min="5" max="5" width="33" customWidth="1"/>
+    <col min="6" max="6" width="17.88671875" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" customWidth="1"/>
+    <col min="9" max="9" width="44.44140625" customWidth="1"/>
+    <col min="10" max="10" width="31.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="23.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="43.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -639,64 +717,124 @@
       <c r="E3" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="F3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="86.4">
       <c r="A4" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3">
+        <v>100000</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="86.4">
       <c r="A5" s="3" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="3">
+        <v>40000</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="H5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="100.8">
       <c r="A6" s="3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="E6" s="3">
+        <v>100000</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="3">
+        <v>2</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="23.4">
       <c r="A8" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="43.2">
       <c r="A10" s="2" t="s">
         <v>1</v>
       </c>
@@ -712,64 +850,124 @@
       <c r="E10" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="F10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="115.2">
       <c r="A11" s="3" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="E11" s="3">
+        <v>999999999</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="100.8">
       <c r="A12" s="3" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="E12" s="3">
+        <v>50000</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="129.6">
       <c r="A13" s="3" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="E13" s="3">
+        <v>40000</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I13" s="3">
+        <v>1</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="23.4">
       <c r="A15" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="43.2">
       <c r="A17" s="2" t="s">
         <v>1</v>
       </c>
@@ -785,73 +983,133 @@
       <c r="E17" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="F17" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="72">
       <c r="A18" s="3" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+      <c r="E18" s="3">
+        <v>-50000</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="72">
       <c r="A19" s="3" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="72">
       <c r="A20" s="3" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="E20" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I20" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="86.4">
       <c r="A21" s="3" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>57</v>
+        <v>66</v>
+      </c>
+      <c r="E21" s="3">
+        <v>100000</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>